<commit_message>
chore: updating game tracker as of 03/04/2026
</commit_message>
<xml_diff>
--- a/public/Game Tracking.xlsx
+++ b/public/Game Tracking.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29816"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shane\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8EA7BA76-7645-4E56-BFA4-B8A25F2E37E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{834CBEA3-E53D-40A4-9924-BB5BB5F3B1C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="1" xr2:uid="{A9AA8E54-3EFE-49B2-8D89-417FC60032EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="4" activeTab="1" xr2:uid="{A9AA8E54-3EFE-49B2-8D89-417FC60032EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Players" sheetId="3" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="156">
   <si>
     <t>PlayerID</t>
   </si>
@@ -442,6 +442,24 @@
     <t>Noctis, Heir Apparent</t>
   </si>
   <si>
+    <t>D40</t>
+  </si>
+  <si>
+    <t>Betor, Ancestor's Voice</t>
+  </si>
+  <si>
+    <t>Cleric Tribal</t>
+  </si>
+  <si>
+    <t>D41</t>
+  </si>
+  <si>
+    <t>Leonardo, The Balance / Donatello, the Brains</t>
+  </si>
+  <si>
+    <t>TMNT</t>
+  </si>
+  <si>
     <t>GameID</t>
   </si>
   <si>
@@ -485,6 +503,15 @@
   </si>
   <si>
     <t>G008</t>
+  </si>
+  <si>
+    <t>G009</t>
+  </si>
+  <si>
+    <t>SpellTable</t>
+  </si>
+  <si>
+    <t>G010</t>
   </si>
   <si>
     <t>Result</t>
@@ -769,8 +796,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{124A738D-4147-4461-B298-69BEE93B2669}" name="tblDecks" displayName="tblDecks" ref="A1:F40" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
-  <autoFilter ref="A1:F40" xr:uid="{124A738D-4147-4461-B298-69BEE93B2669}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{124A738D-4147-4461-B298-69BEE93B2669}" name="tblDecks" displayName="tblDecks" ref="A1:F42" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+  <autoFilter ref="A1:F42" xr:uid="{124A738D-4147-4461-B298-69BEE93B2669}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{A37F2786-4469-4530-B4AF-29BCEDB7309A}" name="DeckID" dataDxfId="17"/>
     <tableColumn id="2" xr3:uid="{F568D9BC-8A66-48EE-B49E-7D58CF2EB57A}" name="PlayerName" dataDxfId="16"/>
@@ -784,8 +811,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}" name="tblGames" displayName="tblGames" ref="A1:E9" totalsRowShown="0" headerRowDxfId="12">
-  <autoFilter ref="A1:E9" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}" name="tblGames" displayName="tblGames" ref="A1:E11" totalsRowShown="0" headerRowDxfId="12">
+  <autoFilter ref="A1:E11" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{3F616AF0-E4FB-4BBD-B459-C9A499225CEE}" name="GameID" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{9AF8C8E1-5799-4D21-A723-4C96DBB5D897}" name="Date" dataDxfId="10"/>
@@ -798,8 +825,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}" name="tblGamePlayers" displayName="tblGamePlayers" ref="A1:F33" totalsRowShown="0" headerRowDxfId="9">
-  <autoFilter ref="A1:F33" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}" name="tblGamePlayers" displayName="tblGamePlayers" ref="A1:F41" totalsRowShown="0" headerRowDxfId="9">
+  <autoFilter ref="A1:F41" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C27C6532-A27F-4D01-B9CF-AE4263247A47}" name="GameID" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{E0277092-F71F-48D5-A8AA-C198C9F208AC}" name="PlayerName"/>
@@ -822,8 +849,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C275F01C-D714-464A-AC0E-262F0026B0CC}" name="Table6" displayName="Table6" ref="A1:G40" totalsRowShown="0" headerRowDxfId="6">
-  <autoFilter ref="A1:G40" xr:uid="{C275F01C-D714-464A-AC0E-262F0026B0CC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C275F01C-D714-464A-AC0E-262F0026B0CC}" name="Table6" displayName="Table6" ref="A1:G42" totalsRowShown="0" headerRowDxfId="6">
+  <autoFilter ref="A1:G42" xr:uid="{C275F01C-D714-464A-AC0E-262F0026B0CC}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C933E5F9-F0B5-4154-A1F4-84EC0B10B856}" name="DeckID" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{1852B62A-968C-4A7A-8FBB-4242180FE226}" name="Commander" dataDxfId="4">
@@ -1247,7 +1274,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6C300ED-5CE2-4173-8CC1-6890A7CDF6C4}">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.140625" customWidth="1"/>
@@ -1930,6 +1957,40 @@
         <v>19781450</v>
       </c>
     </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="F41" s="2">
+        <v>18183110</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="29.25">
+      <c r="A42" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F42" s="2">
+        <v>20391846</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1941,7 +2002,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D73DA2-4E88-40A0-A474-F04E2F001FAF}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" customWidth="1"/>
@@ -1953,30 +2014,30 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30">
       <c r="A2" s="2" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B2" s="4">
         <v>46071</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D2" s="2">
         <v>4</v>
@@ -1985,30 +2046,30 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B3" s="4">
         <v>46071</v>
       </c>
       <c r="C3" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D3">
         <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B4" s="4">
         <v>46072</v>
       </c>
       <c r="C4" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D4">
         <v>4</v>
@@ -2016,13 +2077,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B5" s="4">
         <v>46072</v>
       </c>
       <c r="C5" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D5">
         <v>4</v>
@@ -2030,13 +2091,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B6" s="4">
         <v>46072</v>
       </c>
       <c r="C6" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -2044,13 +2105,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B7" s="4">
         <v>46075</v>
       </c>
       <c r="C7" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -2058,13 +2119,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B8" s="4">
         <v>46075</v>
       </c>
       <c r="C8" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D8">
         <v>4</v>
@@ -2072,15 +2133,43 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B9" s="4">
         <v>46075</v>
       </c>
       <c r="C9" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B10" s="4">
+        <v>46085</v>
+      </c>
+      <c r="C10" t="s">
+        <v>146</v>
+      </c>
+      <c r="D10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B11" s="4">
+        <v>46085</v>
+      </c>
+      <c r="C11" t="s">
+        <v>136</v>
+      </c>
+      <c r="D11">
         <v>4</v>
       </c>
     </row>
@@ -2095,7 +2184,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{901B77E3-1F91-4E2B-8B00-0170C6CF2EFB}">
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" customWidth="1"/>
@@ -2107,7 +2196,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -2119,15 +2208,15 @@
         <v>17</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
@@ -2145,7 +2234,7 @@
         <v>37</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F2" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2154,7 +2243,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="2" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>11</v>
@@ -2172,7 +2261,7 @@
         <v>104</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F3" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2181,7 +2270,7 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>9</v>
@@ -2199,7 +2288,7 @@
         <v>69</v>
       </c>
       <c r="E4" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="F4" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2208,7 +2297,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="2" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>5</v>
@@ -2226,7 +2315,7 @@
         <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F5" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2235,7 +2324,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>3</v>
@@ -2253,7 +2342,7 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F6" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2262,7 +2351,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>11</v>
@@ -2280,7 +2369,7 @@
         <v>107</v>
       </c>
       <c r="E7" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F7" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2289,7 +2378,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>9</v>
@@ -2307,7 +2396,7 @@
         <v>76</v>
       </c>
       <c r="E8" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F8" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2316,7 +2405,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>5</v>
@@ -2334,7 +2423,7 @@
         <v>66</v>
       </c>
       <c r="E9" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="F9" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2343,7 +2432,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="2" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B10" t="s">
         <v>5</v>
@@ -2361,7 +2450,7 @@
         <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="F10" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2370,7 +2459,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="2" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B11" t="s">
         <v>13</v>
@@ -2388,7 +2477,7 @@
         <v>123</v>
       </c>
       <c r="E11" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F11" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2397,7 +2486,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="2" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B12" t="s">
         <v>7</v>
@@ -2415,7 +2504,7 @@
         <v>101</v>
       </c>
       <c r="E12" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F12" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2424,7 +2513,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="2" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B13" t="s">
         <v>9</v>
@@ -2442,7 +2531,7 @@
         <v>80</v>
       </c>
       <c r="E13" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F13" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2451,7 +2540,7 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
@@ -2469,7 +2558,7 @@
         <v>74</v>
       </c>
       <c r="E14" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F14" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2478,7 +2567,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B15" t="s">
         <v>7</v>
@@ -2496,7 +2585,7 @@
         <v>101</v>
       </c>
       <c r="E15" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="F15" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2505,7 +2594,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B16" t="s">
         <v>13</v>
@@ -2523,7 +2612,7 @@
         <v>123</v>
       </c>
       <c r="E16" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F16" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2532,7 +2621,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B17" t="s">
         <v>11</v>
@@ -2550,7 +2639,7 @@
         <v>104</v>
       </c>
       <c r="E17" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F17" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2559,7 +2648,7 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B18" t="s">
         <v>7</v>
@@ -2577,7 +2666,7 @@
         <v>89</v>
       </c>
       <c r="E18" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="F18" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2586,7 +2675,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B19" t="s">
         <v>9</v>
@@ -2604,7 +2693,7 @@
         <v>71</v>
       </c>
       <c r="E19" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F19" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2613,7 +2702,7 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B20" t="s">
         <v>13</v>
@@ -2631,7 +2720,7 @@
         <v>123</v>
       </c>
       <c r="E20" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F20" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2640,7 +2729,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B21" t="s">
         <v>11</v>
@@ -2658,7 +2747,7 @@
         <v>58</v>
       </c>
       <c r="E21" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F21" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2667,7 +2756,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="2" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B22" t="s">
         <v>3</v>
@@ -2685,7 +2774,7 @@
         <v>34</v>
       </c>
       <c r="E22" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F22" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2694,7 +2783,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="2" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B23" t="s">
         <v>5</v>
@@ -2712,7 +2801,7 @@
         <v>54</v>
       </c>
       <c r="E23" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="F23" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2721,7 +2810,7 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="2" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B24" t="s">
         <v>11</v>
@@ -2739,7 +2828,7 @@
         <v>104</v>
       </c>
       <c r="E24" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F24" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2748,7 +2837,7 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="2" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B25" t="s">
         <v>9</v>
@@ -2766,7 +2855,7 @@
         <v>83</v>
       </c>
       <c r="E25" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F25" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2775,7 +2864,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="2" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B26" t="s">
         <v>3</v>
@@ -2793,7 +2882,7 @@
         <v>31</v>
       </c>
       <c r="E26" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="F26" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2802,7 +2891,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="2" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B27" t="s">
         <v>9</v>
@@ -2820,7 +2909,7 @@
         <v>78</v>
       </c>
       <c r="E27" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F27" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2829,7 +2918,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="2" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B28" t="s">
         <v>13</v>
@@ -2847,7 +2936,7 @@
         <v>123</v>
       </c>
       <c r="E28" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F28" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2856,7 +2945,7 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="2" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B29" t="s">
         <v>11</v>
@@ -2874,7 +2963,7 @@
         <v>107</v>
       </c>
       <c r="E29" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F29" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2883,7 +2972,7 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="2" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B30" t="s">
         <v>5</v>
@@ -2901,7 +2990,7 @@
         <v>56</v>
       </c>
       <c r="E30" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="F30" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2910,7 +2999,7 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="2" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B31" t="s">
         <v>7</v>
@@ -2928,7 +3017,7 @@
         <v>86</v>
       </c>
       <c r="E31" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F31" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2937,7 +3026,7 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="2" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B32" t="s">
         <v>11</v>
@@ -2955,7 +3044,7 @@
         <v>58</v>
       </c>
       <c r="E32" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F32" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2964,7 +3053,7 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="2" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B33" t="s">
         <v>9</v>
@@ -2982,9 +3071,225 @@
         <v>71</v>
       </c>
       <c r="E33" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F33" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B34" t="s">
+        <v>3</v>
+      </c>
+      <c r="C34" t="str" cm="1">
+        <f t="array" ref="C34">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D40</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E34" t="s">
+        <v>150</v>
+      </c>
+      <c r="F34" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" t="str" cm="1">
+        <f t="array" ref="C35">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D41</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="E35" t="s">
+        <v>150</v>
+      </c>
+      <c r="F35" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B36" t="s">
+        <v>11</v>
+      </c>
+      <c r="C36" t="str" cm="1">
+        <f t="array" ref="C36">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D31</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E36" t="s">
+        <v>150</v>
+      </c>
+      <c r="F36" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B37" t="s">
+        <v>5</v>
+      </c>
+      <c r="C37" t="str" cm="1">
+        <f t="array" ref="C37">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D10</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E37" t="s">
+        <v>151</v>
+      </c>
+      <c r="F37" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B38" t="s">
+        <v>3</v>
+      </c>
+      <c r="C38" t="str" cm="1">
+        <f t="array" ref="C38">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D40</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E38" t="s">
+        <v>150</v>
+      </c>
+      <c r="F38" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B39" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" t="str" cm="1">
+        <f t="array" ref="C39">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D41</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="E39" t="s">
+        <v>150</v>
+      </c>
+      <c r="F39" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B40" t="s">
+        <v>5</v>
+      </c>
+      <c r="C40" t="str" cm="1">
+        <f t="array" ref="C40">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D15</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E40" t="s">
+        <v>151</v>
+      </c>
+      <c r="F40" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B41" t="s">
+        <v>11</v>
+      </c>
+      <c r="C41" t="str" cm="1">
+        <f t="array" ref="C41">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D32</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E41" t="s">
+        <v>150</v>
+      </c>
+      <c r="F41" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
         <v>0</v>
       </c>
@@ -2992,10 +3297,10 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B33" xr:uid="{8681415D-26E5-48F3-B990-4324A23F1CFB}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B41" xr:uid="{8681415D-26E5-48F3-B990-4324A23F1CFB}">
       <formula1>PlayerList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D33" xr:uid="{9AB3173F-ADED-4CC0-9DF0-944D59BAC803}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D41" xr:uid="{9AB3173F-ADED-4CC0-9DF0-944D59BAC803}">
       <formula1>CommanderList</formula1>
     </dataValidation>
   </dataValidations>
@@ -3008,7 +3313,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2FAD5EF-FA4E-4366-BDF6-EE476BE4A0C0}">
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.7109375" customWidth="1"/>
@@ -3030,16 +3335,16 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -3317,11 +3622,11 @@
       </c>
       <c r="D11">
         <f>COUNTIF(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11">
         <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Win")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11">
         <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss")</f>
@@ -3329,7 +3634,7 @@
       </c>
       <c r="G11" s="6">
         <f>IF(Table6[[#This Row],[Total Games]]=0,0,Table6[[#This Row],[Wins]]/Table6[[#This Row],[Total Games]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -3462,11 +3767,11 @@
       </c>
       <c r="D16">
         <f>COUNTIF(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16">
         <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Win")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16">
         <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss")</f>
@@ -3474,7 +3779,7 @@
       </c>
       <c r="G16" s="6">
         <f>IF(Table6[[#This Row],[Total Games]]=0,0,Table6[[#This Row],[Wins]]/Table6[[#This Row],[Total Games]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -3924,7 +4229,7 @@
       </c>
       <c r="D32">
         <f>COUNTIF(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32">
         <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Win")</f>
@@ -3932,7 +4237,7 @@
       </c>
       <c r="F32">
         <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G32" s="6">
         <f>IF(Table6[[#This Row],[Total Games]]=0,0,Table6[[#This Row],[Wins]]/Table6[[#This Row],[Total Games]])</f>
@@ -3953,7 +4258,7 @@
       </c>
       <c r="D33">
         <f>COUNTIF(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]])</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E33">
         <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Win")</f>
@@ -3961,7 +4266,7 @@
       </c>
       <c r="F33">
         <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G33" s="6">
         <f>IF(Table6[[#This Row],[Total Games]]=0,0,Table6[[#This Row],[Wins]]/Table6[[#This Row],[Total Games]])</f>
@@ -4087,26 +4392,27 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B38" s="7" t="str">
+        <v>116</v>
+      </c>
+      <c r="B38" t="str">
         <f>_xlfn.XLOOKUP(Table6[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[Commander], "")</f>
-        <v>Noctis, Heir Apparent</v>
-      </c>
-      <c r="C38" s="7" t="str">
+        <v>Eluge, the Shoreless Sea</v>
+      </c>
+      <c r="C38" t="str">
         <f>_xlfn.XLOOKUP(Table6[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[PlayerName], "")</f>
-        <v>Franklin</v>
+        <v>Jon Paul</v>
       </c>
       <c r="D38">
         <f>COUNTIF(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]])</f>
-        <v>4</v>
-      </c>
-      <c r="E38" s="7">
+        <v>0</v>
+      </c>
+      <c r="E38">
         <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Win")</f>
         <v>0</v>
       </c>
-      <c r="F38" s="7">
-        <v>3</v>
+      <c r="F38">
+        <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss")</f>
+        <v>0</v>
       </c>
       <c r="G38" s="6">
         <f>IF(Table6[[#This Row],[Total Games]]=0,0,Table6[[#This Row],[Wins]]/Table6[[#This Row],[Total Games]])</f>
@@ -4115,11 +4421,11 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B39" t="str">
         <f>_xlfn.XLOOKUP(Table6[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[Commander], "")</f>
-        <v>Eluge, the Shoreless Sea</v>
+        <v>Ms. Bumbleflower</v>
       </c>
       <c r="C39" t="str">
         <f>_xlfn.XLOOKUP(Table6[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[PlayerName], "")</f>
@@ -4144,19 +4450,19 @@
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B40" t="str">
         <f>_xlfn.XLOOKUP(Table6[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[Commander], "")</f>
-        <v>Ms. Bumbleflower</v>
+        <v>Noctis, Heir Apparent</v>
       </c>
       <c r="C40" t="str">
         <f>_xlfn.XLOOKUP(Table6[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[PlayerName], "")</f>
-        <v>Jon Paul</v>
+        <v>Franklin</v>
       </c>
       <c r="D40">
         <f>COUNTIF(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E40">
         <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Win")</f>
@@ -4164,9 +4470,67 @@
       </c>
       <c r="F40">
         <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G40" s="6">
+        <f>IF(Table6[[#This Row],[Total Games]]=0,0,Table6[[#This Row],[Wins]]/Table6[[#This Row],[Total Games]])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B41" t="str">
+        <f>_xlfn.XLOOKUP(Table6[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[Commander], "")</f>
+        <v>Betor, Ancestor's Voice</v>
+      </c>
+      <c r="C41" t="str">
+        <f>_xlfn.XLOOKUP(Table6[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[PlayerName], "")</f>
+        <v>Shane</v>
+      </c>
+      <c r="D41">
+        <f>COUNTIF(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]])</f>
+        <v>2</v>
+      </c>
+      <c r="E41">
+        <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Win")</f>
+        <v>0</v>
+      </c>
+      <c r="F41">
+        <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss")</f>
+        <v>2</v>
+      </c>
+      <c r="G41" s="6">
+        <f>IF(Table6[[#This Row],[Total Games]]=0,0,Table6[[#This Row],[Wins]]/Table6[[#This Row],[Total Games]])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B42" t="str">
+        <f>_xlfn.XLOOKUP(Table6[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[Commander], "")</f>
+        <v>Leonardo, The Balance / Donatello, the Brains</v>
+      </c>
+      <c r="C42" t="str">
+        <f>_xlfn.XLOOKUP(Table6[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[PlayerName], "")</f>
+        <v>Chavez</v>
+      </c>
+      <c r="D42">
+        <f>COUNTIF(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]])</f>
+        <v>2</v>
+      </c>
+      <c r="E42">
+        <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Win")</f>
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <f>COUNTIFS(tblGamePlayers[DeckID],Table6[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss")</f>
+        <v>2</v>
+      </c>
+      <c r="G42" s="6">
         <f>IF(Table6[[#This Row],[Total Games]]=0,0,Table6[[#This Row],[Wins]]/Table6[[#This Row],[Total Games]])</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
chore: updating game tracker as of 03/26/2026
</commit_message>
<xml_diff>
--- a/public/Game Tracking.xlsx
+++ b/public/Game Tracking.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29917"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shane\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3BA80CBC-99A8-481C-9223-0056E7755CED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7602E36-9196-45B0-B88D-3EC5795D6080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{A9AA8E54-3EFE-49B2-8D89-417FC60032EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A9AA8E54-3EFE-49B2-8D89-417FC60032EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Players" sheetId="3" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="183">
   <si>
     <t>PlayerID</t>
   </si>
@@ -586,6 +586,18 @@
     <t>G017</t>
   </si>
   <si>
+    <t>G018</t>
+  </si>
+  <si>
+    <t>G019</t>
+  </si>
+  <si>
+    <t>G020</t>
+  </si>
+  <si>
+    <t>G021</t>
+  </si>
+  <si>
     <t>Result</t>
   </si>
   <si>
@@ -596,9 +608,6 @@
   </si>
   <si>
     <t>Win</t>
-  </si>
-  <si>
-    <t>G018</t>
   </si>
   <si>
     <t>Total Games</t>
@@ -907,8 +916,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}" name="tblGames" displayName="tblGames" ref="A1:E19" totalsRowShown="0" headerRowDxfId="12">
-  <autoFilter ref="A1:E19" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}" name="tblGames" displayName="tblGames" ref="A1:E22" totalsRowShown="0" headerRowDxfId="12">
+  <autoFilter ref="A1:E22" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{3F616AF0-E4FB-4BBD-B459-C9A499225CEE}" name="GameID" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{9AF8C8E1-5799-4D21-A723-4C96DBB5D897}" name="Date" dataDxfId="10"/>
@@ -921,8 +930,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}" name="tblGamePlayers" displayName="tblGamePlayers" ref="A1:F73" totalsRowShown="0" headerRowDxfId="9">
-  <autoFilter ref="A1:F73" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}" name="tblGamePlayers" displayName="tblGamePlayers" ref="A1:F85" totalsRowShown="0" headerRowDxfId="9">
+  <autoFilter ref="A1:F85" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C27C6532-A27F-4D01-B9CF-AE4263247A47}" name="GameID" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{E0277092-F71F-48D5-A8AA-C198C9F208AC}" name="PlayerName"/>
@@ -1323,7 +1332,7 @@
       </c>
       <c r="C2" s="2">
         <f>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D2" s="2">
         <f>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
@@ -1331,7 +1340,7 @@
       </c>
       <c r="E2" s="8">
         <f>IF(tblPlayers[[#This Row],[GamesPlayed]]=0,0,tblPlayers[[#This Row],[Wins]]/tblPlayers[[#This Row],[GamesPlayed]])</f>
-        <v>0.16666666666666666</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1343,15 +1352,15 @@
       </c>
       <c r="C3" s="2">
         <f>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D3" s="2">
         <f>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E3" s="8">
         <f>IF(tblPlayers[[#This Row],[GamesPlayed]]=0,0,tblPlayers[[#This Row],[Wins]]/tblPlayers[[#This Row],[GamesPlayed]])</f>
-        <v>0.6428571428571429</v>
+        <v>0.6875</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1383,7 +1392,7 @@
       </c>
       <c r="C5" s="2">
         <f>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D5" s="2">
         <f>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
@@ -1391,7 +1400,7 @@
       </c>
       <c r="E5" s="8">
         <f>IF(tblPlayers[[#This Row],[GamesPlayed]]=0,0,tblPlayers[[#This Row],[Wins]]/tblPlayers[[#This Row],[GamesPlayed]])</f>
-        <v>0.17647058823529413</v>
+        <v>0.14285714285714285</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1403,15 +1412,15 @@
       </c>
       <c r="C6" s="2">
         <f>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D6" s="2">
         <f>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6" s="8">
         <f>IF(tblPlayers[[#This Row],[GamesPlayed]]=0,0,tblPlayers[[#This Row],[Wins]]/tblPlayers[[#This Row],[GamesPlayed]])</f>
-        <v>6.25E-2</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1443,7 +1452,7 @@
       </c>
       <c r="C8" s="2">
         <f>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D8" s="2">
         <f>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
@@ -2312,7 +2321,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D73DA2-4E88-40A0-A474-F04E2F001FAF}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" customWidth="1"/>
@@ -2585,8 +2594,60 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="2"/>
-      <c r="B19" s="4"/>
+      <c r="A19" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B19" s="4">
+        <v>46095</v>
+      </c>
+      <c r="C19" t="s">
+        <v>151</v>
+      </c>
+      <c r="D19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B20" s="4">
+        <v>46095</v>
+      </c>
+      <c r="C20" t="s">
+        <v>151</v>
+      </c>
+      <c r="D20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B21" s="4">
+        <v>46105</v>
+      </c>
+      <c r="C21" t="s">
+        <v>151</v>
+      </c>
+      <c r="D21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B22" s="4">
+        <v>46106</v>
+      </c>
+      <c r="C22" t="s">
+        <v>151</v>
+      </c>
+      <c r="D22">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -2599,7 +2660,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{901B77E3-1F91-4E2B-8B00-0170C6CF2EFB}">
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" customWidth="1"/>
@@ -2623,10 +2684,10 @@
         <v>20</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2649,7 +2710,7 @@
         <v>40</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F2" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2676,7 +2737,7 @@
         <v>107</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F3" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2703,7 +2764,7 @@
         <v>72</v>
       </c>
       <c r="E4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F4" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2730,7 +2791,7 @@
         <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F5" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2757,7 +2818,7 @@
         <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F6" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2784,7 +2845,7 @@
         <v>110</v>
       </c>
       <c r="E7" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F7" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2811,7 +2872,7 @@
         <v>79</v>
       </c>
       <c r="E8" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F8" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2838,7 +2899,7 @@
         <v>69</v>
       </c>
       <c r="E9" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F9" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2865,7 +2926,7 @@
         <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F10" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2892,7 +2953,7 @@
         <v>126</v>
       </c>
       <c r="E11" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F11" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2919,7 +2980,7 @@
         <v>104</v>
       </c>
       <c r="E12" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F12" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2946,7 +3007,7 @@
         <v>83</v>
       </c>
       <c r="E13" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F13" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2973,7 +3034,7 @@
         <v>77</v>
       </c>
       <c r="E14" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F14" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3000,7 +3061,7 @@
         <v>104</v>
       </c>
       <c r="E15" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F15" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3027,7 +3088,7 @@
         <v>126</v>
       </c>
       <c r="E16" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F16" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3054,7 +3115,7 @@
         <v>107</v>
       </c>
       <c r="E17" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F17" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3081,7 +3142,7 @@
         <v>92</v>
       </c>
       <c r="E18" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F18" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3108,7 +3169,7 @@
         <v>74</v>
       </c>
       <c r="E19" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F19" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3135,7 +3196,7 @@
         <v>126</v>
       </c>
       <c r="E20" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F20" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3162,7 +3223,7 @@
         <v>61</v>
       </c>
       <c r="E21" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F21" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3189,7 +3250,7 @@
         <v>37</v>
       </c>
       <c r="E22" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F22" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3216,7 +3277,7 @@
         <v>57</v>
       </c>
       <c r="E23" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F23" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3243,7 +3304,7 @@
         <v>107</v>
       </c>
       <c r="E24" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F24" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3270,7 +3331,7 @@
         <v>86</v>
       </c>
       <c r="E25" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F25" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3297,7 +3358,7 @@
         <v>34</v>
       </c>
       <c r="E26" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F26" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3324,7 +3385,7 @@
         <v>81</v>
       </c>
       <c r="E27" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F27" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3351,7 +3412,7 @@
         <v>126</v>
       </c>
       <c r="E28" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F28" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3378,7 +3439,7 @@
         <v>110</v>
       </c>
       <c r="E29" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F29" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3405,7 +3466,7 @@
         <v>59</v>
       </c>
       <c r="E30" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F30" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3432,7 +3493,7 @@
         <v>89</v>
       </c>
       <c r="E31" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F31" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3459,7 +3520,7 @@
         <v>61</v>
       </c>
       <c r="E32" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F32" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3486,7 +3547,7 @@
         <v>74</v>
       </c>
       <c r="E33" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F33" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3513,7 +3574,7 @@
         <v>128</v>
       </c>
       <c r="E34" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F34" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3540,7 +3601,7 @@
         <v>131</v>
       </c>
       <c r="E35" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F35" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3567,7 +3628,7 @@
         <v>107</v>
       </c>
       <c r="E36" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F36" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3594,7 +3655,7 @@
         <v>52</v>
       </c>
       <c r="E37" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F37" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3621,7 +3682,7 @@
         <v>128</v>
       </c>
       <c r="E38" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F38" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3648,7 +3709,7 @@
         <v>131</v>
       </c>
       <c r="E39" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F39" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3675,7 +3736,7 @@
         <v>64</v>
       </c>
       <c r="E40" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F40" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3702,7 +3763,7 @@
         <v>110</v>
       </c>
       <c r="E41" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F41" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3729,7 +3790,7 @@
         <v>95</v>
       </c>
       <c r="E42" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F42" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3756,7 +3817,7 @@
         <v>131</v>
       </c>
       <c r="E43" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F43" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3783,7 +3844,7 @@
         <v>57</v>
       </c>
       <c r="E44" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F44" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3810,7 +3871,7 @@
         <v>107</v>
       </c>
       <c r="E45" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F45" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3837,7 +3898,7 @@
         <v>98</v>
       </c>
       <c r="E46" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F46" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3864,7 +3925,7 @@
         <v>77</v>
       </c>
       <c r="E47" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F47" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3891,7 +3952,7 @@
         <v>134</v>
       </c>
       <c r="E48" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F48" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3918,7 +3979,7 @@
         <v>110</v>
       </c>
       <c r="E49" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F49" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3945,7 +4006,7 @@
         <v>89</v>
       </c>
       <c r="E50" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F50" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3972,7 +4033,7 @@
         <v>74</v>
       </c>
       <c r="E51" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F51" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3999,7 +4060,7 @@
         <v>59</v>
       </c>
       <c r="E52" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F52" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4026,7 +4087,7 @@
         <v>114</v>
       </c>
       <c r="E53" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F53" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4053,7 +4114,7 @@
         <v>89</v>
       </c>
       <c r="E54" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F54" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4080,7 +4141,7 @@
         <v>72</v>
       </c>
       <c r="E55" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F55" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4107,7 +4168,7 @@
         <v>59</v>
       </c>
       <c r="E56" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F56" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4134,7 +4195,7 @@
         <v>114</v>
       </c>
       <c r="E57" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F57" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4161,7 +4222,7 @@
         <v>137</v>
       </c>
       <c r="E58" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F58" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4188,7 +4249,7 @@
         <v>137</v>
       </c>
       <c r="E59" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F59" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4215,7 +4276,7 @@
         <v>52</v>
       </c>
       <c r="E60" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F60" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4242,7 +4303,7 @@
         <v>114</v>
       </c>
       <c r="E61" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F61" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4269,7 +4330,7 @@
         <v>137</v>
       </c>
       <c r="E62" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F62" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4296,7 +4357,7 @@
         <v>131</v>
       </c>
       <c r="E63" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F63" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4323,7 +4384,7 @@
         <v>137</v>
       </c>
       <c r="E64" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F64" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4350,7 +4411,7 @@
         <v>61</v>
       </c>
       <c r="E65" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F65" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4377,7 +4438,7 @@
         <v>104</v>
       </c>
       <c r="E66" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F66" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4404,7 +4465,7 @@
         <v>81</v>
       </c>
       <c r="E67" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F67" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4431,7 +4492,7 @@
         <v>61</v>
       </c>
       <c r="E68" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F68" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4458,7 +4519,7 @@
         <v>110</v>
       </c>
       <c r="E69" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="F69" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4467,7 +4528,10 @@
     </row>
     <row r="70" spans="1:6">
       <c r="A70" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
+      </c>
+      <c r="B70" t="s">
+        <v>12</v>
       </c>
       <c r="C70" t="str" cm="1">
         <f t="array" ref="C70">_xlfn.XLOOKUP(1,
@@ -4476,9 +4540,14 @@
    tblDecks[DeckID],
    ""
 )</f>
-        <v/>
-      </c>
-      <c r="D70" s="7"/>
+        <v>D41</v>
+      </c>
+      <c r="D70" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="E70" t="s">
+        <v>178</v>
+      </c>
       <c r="F70" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
         <v>0</v>
@@ -4486,7 +4555,10 @@
     </row>
     <row r="71" spans="1:6">
       <c r="A71" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
+      </c>
+      <c r="B71" t="s">
+        <v>6</v>
       </c>
       <c r="C71" t="str" cm="1">
         <f t="array" ref="C71">_xlfn.XLOOKUP(1,
@@ -4495,9 +4567,14 @@
    tblDecks[DeckID],
    ""
 )</f>
-        <v/>
-      </c>
-      <c r="D71" s="7"/>
+        <v>D40</v>
+      </c>
+      <c r="D71" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="E71" t="s">
+        <v>178</v>
+      </c>
       <c r="F71" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
         <v>0</v>
@@ -4505,7 +4582,10 @@
     </row>
     <row r="72" spans="1:6">
       <c r="A72" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
+      </c>
+      <c r="B72" t="s">
+        <v>14</v>
       </c>
       <c r="C72" t="str" cm="1">
         <f t="array" ref="C72">_xlfn.XLOOKUP(1,
@@ -4514,9 +4594,14 @@
    tblDecks[DeckID],
    ""
 )</f>
-        <v/>
-      </c>
-      <c r="D72" s="7"/>
+        <v>D31</v>
+      </c>
+      <c r="D72" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E72" t="s">
+        <v>178</v>
+      </c>
       <c r="F72" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
         <v>0</v>
@@ -4524,7 +4609,10 @@
     </row>
     <row r="73" spans="1:6">
       <c r="A73" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
+      </c>
+      <c r="B73" t="s">
+        <v>8</v>
       </c>
       <c r="C73" t="str" cm="1">
         <f t="array" ref="C73">_xlfn.XLOOKUP(1,
@@ -4533,18 +4621,347 @@
    tblDecks[DeckID],
    ""
 )</f>
-        <v/>
-      </c>
-      <c r="D73" s="7"/>
+        <v>D16</v>
+      </c>
+      <c r="D73" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="E73" t="s">
+        <v>179</v>
+      </c>
       <c r="F73" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
+      <c r="A74" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B74" t="s">
+        <v>12</v>
+      </c>
+      <c r="C74" t="str" cm="1">
+        <f t="array" ref="C74">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D20</v>
+      </c>
+      <c r="D74" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E74" t="s">
+        <v>178</v>
+      </c>
+      <c r="F74" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
+      <c r="A75" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B75" t="s">
+        <v>6</v>
+      </c>
+      <c r="C75" t="str" cm="1">
+        <f t="array" ref="C75">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D1</v>
+      </c>
+      <c r="D75" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E75" t="s">
+        <v>178</v>
+      </c>
+      <c r="F75" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="A76" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B76" t="s">
+        <v>14</v>
+      </c>
+      <c r="C76" t="str" cm="1">
+        <f t="array" ref="C76">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D33</v>
+      </c>
+      <c r="D76" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E76" t="s">
+        <v>178</v>
+      </c>
+      <c r="F76" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="A77" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B77" t="s">
+        <v>8</v>
+      </c>
+      <c r="C77" t="str" cm="1">
+        <f t="array" ref="C77">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D8</v>
+      </c>
+      <c r="D77" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E77" t="s">
+        <v>179</v>
+      </c>
+      <c r="F77" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
+      <c r="A78" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B78" t="s">
+        <v>6</v>
+      </c>
+      <c r="C78" t="str" cm="1">
+        <f t="array" ref="C78">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D40</v>
+      </c>
+      <c r="D78" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="E78" t="s">
+        <v>178</v>
+      </c>
+      <c r="F78" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
+      <c r="A79" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B79" t="s">
+        <v>14</v>
+      </c>
+      <c r="C79" t="str" cm="1">
+        <f t="array" ref="C79">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D31</v>
+      </c>
+      <c r="D79" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E79" t="s">
+        <v>179</v>
+      </c>
+      <c r="F79" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
+      <c r="A80" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B80" t="s">
+        <v>12</v>
+      </c>
+      <c r="C80" t="str" cm="1">
+        <f t="array" ref="C80">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D18</v>
+      </c>
+      <c r="D80" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E80" t="s">
+        <v>178</v>
+      </c>
+      <c r="F80" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6">
+      <c r="A81" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B81" t="s">
+        <v>18</v>
+      </c>
+      <c r="C81" t="str" cm="1">
+        <f t="array" ref="C81">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D38</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="E81" t="s">
+        <v>178</v>
+      </c>
+      <c r="F81" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6">
+      <c r="A82" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B82" t="s">
+        <v>6</v>
+      </c>
+      <c r="C82" t="str" cm="1">
+        <f t="array" ref="C82">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D1</v>
+      </c>
+      <c r="D82" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E82" t="s">
+        <v>178</v>
+      </c>
+      <c r="F82" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6">
+      <c r="A83" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B83" t="s">
+        <v>12</v>
+      </c>
+      <c r="C83" t="str" cm="1">
+        <f t="array" ref="C83">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D21</v>
+      </c>
+      <c r="D83" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E83" t="s">
+        <v>178</v>
+      </c>
+      <c r="F83" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6">
+      <c r="A84" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B84" t="s">
+        <v>18</v>
+      </c>
+      <c r="C84" t="str" cm="1">
+        <f t="array" ref="C84">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D38</v>
+      </c>
+      <c r="D84" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="E84" t="s">
+        <v>178</v>
+      </c>
+      <c r="F84" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6">
+      <c r="A85" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B85" t="s">
+        <v>14</v>
+      </c>
+      <c r="C85" t="str" cm="1">
+        <f t="array" ref="C85">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D34</v>
+      </c>
+      <c r="D85" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="E85" t="s">
+        <v>179</v>
+      </c>
+      <c r="F85" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B73" xr:uid="{8681415D-26E5-48F3-B990-4324A23F1CFB}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B85" xr:uid="{8681415D-26E5-48F3-B990-4324A23F1CFB}">
       <formula1>PlayerList</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{86E4FB70-4529-47DF-A939-BD41AD4D0FA0}">
@@ -4582,16 +4999,16 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -4608,7 +5025,7 @@
       </c>
       <c r="D2">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -4616,7 +5033,7 @@
       </c>
       <c r="F2">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G2" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -4811,11 +5228,11 @@
       </c>
       <c r="D9">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
@@ -4823,7 +5240,7 @@
       </c>
       <c r="G9" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -5043,11 +5460,11 @@
       </c>
       <c r="D17">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
@@ -5101,7 +5518,7 @@
       </c>
       <c r="D19">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E19">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5109,11 +5526,11 @@
       </c>
       <c r="F19">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -5159,7 +5576,7 @@
       </c>
       <c r="D21">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5167,7 +5584,7 @@
       </c>
       <c r="F21">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G21" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5188,7 +5605,7 @@
       </c>
       <c r="D22">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5196,7 +5613,7 @@
       </c>
       <c r="F22">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5478,19 +5895,19 @@
       </c>
       <c r="D32">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E32">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G32" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0</v>
+        <v>0.14285714285714285</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -5536,7 +5953,7 @@
       </c>
       <c r="D34">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E34">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5544,7 +5961,7 @@
       </c>
       <c r="F34">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G34" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5565,11 +5982,11 @@
       </c>
       <c r="D35">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E35">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
@@ -5577,7 +5994,7 @@
       </c>
       <c r="G35" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -5682,7 +6099,7 @@
       </c>
       <c r="D39">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E39">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5690,7 +6107,7 @@
       </c>
       <c r="F39">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G39" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5740,7 +6157,7 @@
       </c>
       <c r="D41">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E41">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5748,7 +6165,7 @@
       </c>
       <c r="F41">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G41" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5769,7 +6186,7 @@
       </c>
       <c r="D42">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E42">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5777,11 +6194,11 @@
       </c>
       <c r="F42">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G42" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="43" spans="1:8">

</xml_diff>

<commit_message>
chore: updating game tracker as of 04/27/2026
</commit_message>
<xml_diff>
--- a/public/Game Tracking.xlsx
+++ b/public/Game Tracking.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30015"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shane\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7602E36-9196-45B0-B88D-3EC5795D6080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B320B73-D689-45D7-A0F6-C7D6E9A8EBD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A9AA8E54-3EFE-49B2-8D89-417FC60032EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="4" activeTab="4" xr2:uid="{A9AA8E54-3EFE-49B2-8D89-417FC60032EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Players" sheetId="3" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="207">
   <si>
     <t>PlayerID</t>
   </si>
@@ -505,6 +505,42 @@
     <t>D49</t>
   </si>
   <si>
+    <t>D50</t>
+  </si>
+  <si>
+    <t>Mister Negative</t>
+  </si>
+  <si>
+    <t>Life Swap</t>
+  </si>
+  <si>
+    <t>D51</t>
+  </si>
+  <si>
+    <t>Bria, Riptide Rogue</t>
+  </si>
+  <si>
+    <t>Otters</t>
+  </si>
+  <si>
+    <t>D52</t>
+  </si>
+  <si>
+    <t>Dina, Essence Brewer</t>
+  </si>
+  <si>
+    <t>Witherbloom</t>
+  </si>
+  <si>
+    <t>D53</t>
+  </si>
+  <si>
+    <t>Nashi, Moon Sage's Scion</t>
+  </si>
+  <si>
+    <t>Spell Steal</t>
+  </si>
+  <si>
     <t>GameID</t>
   </si>
   <si>
@@ -596,6 +632,42 @@
   </si>
   <si>
     <t>G021</t>
+  </si>
+  <si>
+    <t>G022</t>
+  </si>
+  <si>
+    <t>JP: Valgavoth</t>
+  </si>
+  <si>
+    <t>G023</t>
+  </si>
+  <si>
+    <t>G024</t>
+  </si>
+  <si>
+    <t>G025</t>
+  </si>
+  <si>
+    <t>G026</t>
+  </si>
+  <si>
+    <t>G027</t>
+  </si>
+  <si>
+    <t>Chavez's</t>
+  </si>
+  <si>
+    <t>Isaac: Saruman</t>
+  </si>
+  <si>
+    <t>G028</t>
+  </si>
+  <si>
+    <t>G029</t>
+  </si>
+  <si>
+    <t>G030</t>
   </si>
   <si>
     <t>Result</t>
@@ -701,7 +773,10 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="28">
+    <dxf>
+      <numFmt numFmtId="13" formatCode="0%"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -881,18 +956,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D34C1EB-B3A7-4BED-BD5D-53202B37AABB}" name="tblPlayers" displayName="tblPlayers" ref="A1:E8" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D34C1EB-B3A7-4BED-BD5D-53202B37AABB}" name="tblPlayers" displayName="tblPlayers" ref="A1:E8" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:E8" xr:uid="{6D34C1EB-B3A7-4BED-BD5D-53202B37AABB}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{12F317AB-51F1-45A7-ADED-E87A2200364C}" name="PlayerID" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{88D5D8C3-E760-4339-B742-29D1D7AE85F1}" name="PlayerName" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{276CAFE3-1614-473F-B917-91E8BEEF5EA1}" name="GamesPlayed" dataDxfId="22">
+    <tableColumn id="1" xr3:uid="{12F317AB-51F1-45A7-ADED-E87A2200364C}" name="PlayerID" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{88D5D8C3-E760-4339-B742-29D1D7AE85F1}" name="PlayerName" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{276CAFE3-1614-473F-B917-91E8BEEF5EA1}" name="GamesPlayed" dataDxfId="23">
       <calculatedColumnFormula>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{E6D338DE-2A91-4BBA-93A9-1CC7F5285D40}" name="Wins" dataDxfId="21">
+    <tableColumn id="4" xr3:uid="{E6D338DE-2A91-4BBA-93A9-1CC7F5285D40}" name="Wins" dataDxfId="22">
       <calculatedColumnFormula>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{72245CB6-0B77-4BC9-9C65-FDCC70075FDA}" name="Win%" dataDxfId="20">
+    <tableColumn id="6" xr3:uid="{72245CB6-0B77-4BC9-9C65-FDCC70075FDA}" name="Win%" dataDxfId="21">
       <calculatedColumnFormula>IF(tblPlayers[[#This Row],[GamesPlayed]]=0,0,tblPlayers[[#This Row],[Wins]]/tblPlayers[[#This Row],[GamesPlayed]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -901,26 +976,26 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{124A738D-4147-4461-B298-69BEE93B2669}" name="tblDecks" displayName="tblDecks" ref="A1:F50" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
-  <autoFilter ref="A1:F50" xr:uid="{124A738D-4147-4461-B298-69BEE93B2669}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{124A738D-4147-4461-B298-69BEE93B2669}" name="tblDecks" displayName="tblDecks" ref="A1:F54" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+  <autoFilter ref="A1:F54" xr:uid="{124A738D-4147-4461-B298-69BEE93B2669}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{A37F2786-4469-4530-B4AF-29BCEDB7309A}" name="DeckID" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{F568D9BC-8A66-48EE-B49E-7D58CF2EB57A}" name="PlayerName" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{98820B81-A857-455B-8F1B-F1B67D87CC74}" name="Commander" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{4F06AA0C-60A1-4886-A43B-7BCA0A8634DF}" name="Theme" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{A37F2786-4469-4530-B4AF-29BCEDB7309A}" name="DeckID" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{F568D9BC-8A66-48EE-B49E-7D58CF2EB57A}" name="PlayerName" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{98820B81-A857-455B-8F1B-F1B67D87CC74}" name="Commander" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{4F06AA0C-60A1-4886-A43B-7BCA0A8634DF}" name="Theme" dataDxfId="15"/>
     <tableColumn id="5" xr3:uid="{EEB55A92-7875-4505-9C72-7E8BB3618F42}" name="EstPower"/>
-    <tableColumn id="6" xr3:uid="{AB3B7E9F-5601-420D-97B2-07DC6E67D6BF}" name="ArchidektID" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{AB3B7E9F-5601-420D-97B2-07DC6E67D6BF}" name="ArchidektID" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}" name="tblGames" displayName="tblGames" ref="A1:E22" totalsRowShown="0" headerRowDxfId="12">
-  <autoFilter ref="A1:E22" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}" name="tblGames" displayName="tblGames" ref="A1:E31" totalsRowShown="0" headerRowDxfId="13">
+  <autoFilter ref="A1:E31" xr:uid="{1ADB571D-D4CB-4C8E-9C94-24EF902812FC}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{3F616AF0-E4FB-4BBD-B459-C9A499225CEE}" name="GameID" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{9AF8C8E1-5799-4D21-A723-4C96DBB5D897}" name="Date" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{3F616AF0-E4FB-4BBD-B459-C9A499225CEE}" name="GameID" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{9AF8C8E1-5799-4D21-A723-4C96DBB5D897}" name="Date" dataDxfId="11"/>
     <tableColumn id="3" xr3:uid="{B13D620E-EB98-45B7-8ECB-DF8CCA6D1EE8}" name="Location"/>
     <tableColumn id="4" xr3:uid="{49C3414B-2C9D-4C17-9096-AC7D0B18B97E}" name="TotalPlayers"/>
     <tableColumn id="5" xr3:uid="{D059AADB-99FE-4453-A1C8-315D8AAC89AC}" name="Notes"/>
@@ -930,10 +1005,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}" name="tblGamePlayers" displayName="tblGamePlayers" ref="A1:F85" totalsRowShown="0" headerRowDxfId="9">
-  <autoFilter ref="A1:F85" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}" name="tblGamePlayers" displayName="tblGamePlayers" ref="A1:F121" totalsRowShown="0" headerRowDxfId="10">
+  <autoFilter ref="A1:F121" xr:uid="{D7DF9500-9C94-4D2F-9FE8-DC3C1ADC86B4}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C27C6532-A27F-4D01-B9CF-AE4263247A47}" name="GameID" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{C27C6532-A27F-4D01-B9CF-AE4263247A47}" name="GameID" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{E0277092-F71F-48D5-A8AA-C198C9F208AC}" name="PlayerName"/>
     <tableColumn id="3" xr3:uid="{D0A81E19-20E8-49D5-B4C2-62526DCCFC25}" name="DeckID">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(1,
@@ -943,7 +1018,7 @@
    ""
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{B3156F92-AF12-4F21-B8E5-1A9FB10A5629}" name="Commander" dataDxfId="7">
+    <tableColumn id="4" xr3:uid="{B3156F92-AF12-4F21-B8E5-1A9FB10A5629}" name="Commander" dataDxfId="8">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblGamePlayers[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[Commander], "")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{72F15DC9-FBE8-498D-862D-5DAB67E25E14}" name="Result"/>
@@ -954,26 +1029,26 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C275F01C-D714-464A-AC0E-262F0026B0CC}" name="tblDeckDashboard" displayName="tblDeckDashboard" ref="A1:G50" totalsRowShown="0" headerRowDxfId="6">
-  <autoFilter ref="A1:G50" xr:uid="{C275F01C-D714-464A-AC0E-262F0026B0CC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C275F01C-D714-464A-AC0E-262F0026B0CC}" name="tblDeckDashboard" displayName="tblDeckDashboard" ref="A1:G54" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:G54" xr:uid="{C275F01C-D714-464A-AC0E-262F0026B0CC}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{C933E5F9-F0B5-4154-A1F4-84EC0B10B856}" name="DeckID" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{1852B62A-968C-4A7A-8FBB-4242180FE226}" name="Commander" dataDxfId="4">
+    <tableColumn id="1" xr3:uid="{C933E5F9-F0B5-4154-A1F4-84EC0B10B856}" name="DeckID" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{1852B62A-968C-4A7A-8FBB-4242180FE226}" name="Commander" dataDxfId="5">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblDeckDashboard[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[Commander], "")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{47AB326A-9A36-4FA8-97D9-70E092F74454}" name="PlayerName" dataDxfId="3">
+    <tableColumn id="3" xr3:uid="{47AB326A-9A36-4FA8-97D9-70E092F74454}" name="PlayerName" dataDxfId="4">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tblDeckDashboard[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[PlayerName], "")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{CB156740-E53A-4902-A4BE-ABFE6B13AEA1}" name="Total Games" dataDxfId="2">
+    <tableColumn id="4" xr3:uid="{CB156740-E53A-4902-A4BE-ABFE6B13AEA1}" name="Total Games" dataDxfId="3">
       <calculatedColumnFormula>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{D0BC7C1B-6547-4010-871C-EADEAE8D80EF}" name="Wins" dataDxfId="1">
+    <tableColumn id="5" xr3:uid="{D0BC7C1B-6547-4010-871C-EADEAE8D80EF}" name="Wins" dataDxfId="2">
       <calculatedColumnFormula>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{176CC7A4-26D9-4CC2-9EEF-D16F2472E603}" name="Losses" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{176CC7A4-26D9-4CC2-9EEF-D16F2472E603}" name="Losses" dataDxfId="1">
       <calculatedColumnFormula>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{C11561C3-6AF2-47A0-9401-8EFD40DA3546}" name="Win %" dataCellStyle="Percent">
+    <tableColumn id="7" xr3:uid="{C11561C3-6AF2-47A0-9401-8EFD40DA3546}" name="Win %" dataDxfId="0" dataCellStyle="Percent">
       <calculatedColumnFormula>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1332,15 +1407,15 @@
       </c>
       <c r="C2" s="2">
         <f>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D2" s="2">
         <f>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" s="8">
         <f>IF(tblPlayers[[#This Row],[GamesPlayed]]=0,0,tblPlayers[[#This Row],[Wins]]/tblPlayers[[#This Row],[GamesPlayed]])</f>
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1352,15 +1427,15 @@
       </c>
       <c r="C3" s="2">
         <f>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2">
         <f>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E3" s="8">
         <f>IF(tblPlayers[[#This Row],[GamesPlayed]]=0,0,tblPlayers[[#This Row],[Wins]]/tblPlayers[[#This Row],[GamesPlayed]])</f>
-        <v>0.6875</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1372,7 +1447,7 @@
       </c>
       <c r="C4" s="2">
         <f>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D4" s="2">
         <f>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
@@ -1380,7 +1455,7 @@
       </c>
       <c r="E4" s="8">
         <f>IF(tblPlayers[[#This Row],[GamesPlayed]]=0,0,tblPlayers[[#This Row],[Wins]]/tblPlayers[[#This Row],[GamesPlayed]])</f>
-        <v>0.27272727272727271</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1392,15 +1467,15 @@
       </c>
       <c r="C5" s="2">
         <f>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="D5" s="2">
         <f>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" s="8">
         <f>IF(tblPlayers[[#This Row],[GamesPlayed]]=0,0,tblPlayers[[#This Row],[Wins]]/tblPlayers[[#This Row],[GamesPlayed]])</f>
-        <v>0.14285714285714285</v>
+        <v>0.13333333333333333</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1412,7 +1487,7 @@
       </c>
       <c r="C6" s="2">
         <f>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D6" s="2">
         <f>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
@@ -1420,7 +1495,7 @@
       </c>
       <c r="E6" s="8">
         <f>IF(tblPlayers[[#This Row],[GamesPlayed]]=0,0,tblPlayers[[#This Row],[Wins]]/tblPlayers[[#This Row],[GamesPlayed]])</f>
-        <v>0.15</v>
+        <v>0.10344827586206896</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1452,15 +1527,15 @@
       </c>
       <c r="C8" s="2">
         <f>COUNTIF(tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D8" s="2">
         <f>SUMIFS(tblGamePlayers[WinFlag],tblGamePlayers[PlayerName],tblPlayers[[#This Row],[PlayerName]])</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E8" s="8">
         <f>IF(tblPlayers[[#This Row],[GamesPlayed]]=0,0,tblPlayers[[#This Row],[Wins]]/tblPlayers[[#This Row],[GamesPlayed]])</f>
-        <v>0</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
   </sheetData>
@@ -1473,7 +1548,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6C300ED-5CE2-4173-8CC1-6890A7CDF6C4}">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.140625" customWidth="1"/>
@@ -2310,6 +2385,66 @@
       </c>
       <c r="F50" s="2"/>
     </row>
+    <row r="51" spans="1:6">
+      <c r="A51" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F51" s="2"/>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F52" s="2"/>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F53" s="2"/>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F54" s="2"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2321,7 +2456,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D73DA2-4E88-40A0-A474-F04E2F001FAF}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" customWidth="1"/>
@@ -2333,30 +2468,30 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B2" s="4">
         <v>46071</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D2" s="2">
         <v>4</v>
@@ -2365,13 +2500,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B3" s="4">
         <v>46071</v>
       </c>
       <c r="C3" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D3">
         <v>4</v>
@@ -2379,13 +2514,13 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B4" s="4">
         <v>46072</v>
       </c>
       <c r="C4" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D4">
         <v>4</v>
@@ -2393,13 +2528,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B5" s="4">
         <v>46072</v>
       </c>
       <c r="C5" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D5">
         <v>4</v>
@@ -2407,13 +2542,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B6" s="4">
         <v>46072</v>
       </c>
       <c r="C6" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -2421,13 +2556,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="B7" s="4">
         <v>46075</v>
       </c>
       <c r="C7" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -2435,13 +2570,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="B8" s="4">
         <v>46075</v>
       </c>
       <c r="C8" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D8">
         <v>4</v>
@@ -2449,13 +2584,13 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="B9" s="4">
         <v>46075</v>
       </c>
       <c r="C9" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D9">
         <v>4</v>
@@ -2463,13 +2598,13 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="B10" s="4">
         <v>46085</v>
       </c>
       <c r="C10" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="D10">
         <v>4</v>
@@ -2477,13 +2612,13 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="B11" s="4">
         <v>46085</v>
       </c>
       <c r="C11" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D11">
         <v>4</v>
@@ -2491,13 +2626,13 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="B12" s="4">
         <v>46088</v>
       </c>
       <c r="C12" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="D12">
         <v>4</v>
@@ -2505,13 +2640,13 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B13" s="4">
         <v>46088</v>
       </c>
       <c r="C13" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="D13">
         <v>4</v>
@@ -2519,13 +2654,13 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B14" s="4">
         <v>46088</v>
       </c>
       <c r="C14" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="D14">
         <v>4</v>
@@ -2533,13 +2668,13 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="B15" s="4">
         <v>46088</v>
       </c>
       <c r="C15" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="D15">
         <v>4</v>
@@ -2547,47 +2682,47 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="B16" s="4">
         <v>46088</v>
       </c>
       <c r="C16" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="D16">
         <v>4</v>
       </c>
       <c r="E16" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="B17" s="4">
         <v>46088</v>
       </c>
       <c r="C17" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="D17">
         <v>4</v>
       </c>
       <c r="E17" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="B18" s="4">
         <v>46088</v>
       </c>
       <c r="C18" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="D18">
         <v>4</v>
@@ -2595,13 +2730,13 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="B19" s="4">
         <v>46095</v>
       </c>
       <c r="C19" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D19">
         <v>4</v>
@@ -2609,13 +2744,13 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="B20" s="4">
         <v>46095</v>
       </c>
       <c r="C20" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D20">
         <v>4</v>
@@ -2623,13 +2758,13 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="B21" s="4">
         <v>46105</v>
       </c>
       <c r="C21" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D21">
         <v>4</v>
@@ -2637,16 +2772,151 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="B22" s="4">
-        <v>46106</v>
+        <v>46105</v>
       </c>
       <c r="C22" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D22">
-        <v>5</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B23" s="4">
+        <v>46112</v>
+      </c>
+      <c r="C23" t="s">
+        <v>163</v>
+      </c>
+      <c r="D23">
+        <v>4</v>
+      </c>
+      <c r="E23" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B24" s="4">
+        <v>46112</v>
+      </c>
+      <c r="C24" t="s">
+        <v>163</v>
+      </c>
+      <c r="D24">
+        <v>4</v>
+      </c>
+      <c r="E24" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B25" s="4">
+        <v>46122</v>
+      </c>
+      <c r="C25" t="s">
+        <v>163</v>
+      </c>
+      <c r="D25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B26" s="4">
+        <v>46122</v>
+      </c>
+      <c r="C26" t="s">
+        <v>163</v>
+      </c>
+      <c r="D26">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B27" s="4">
+        <v>46122</v>
+      </c>
+      <c r="C27" t="s">
+        <v>163</v>
+      </c>
+      <c r="D27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B28" s="4">
+        <v>46136</v>
+      </c>
+      <c r="C28" t="s">
+        <v>195</v>
+      </c>
+      <c r="D28">
+        <v>4</v>
+      </c>
+      <c r="E28" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B29" s="4">
+        <v>46136</v>
+      </c>
+      <c r="C29" t="s">
+        <v>195</v>
+      </c>
+      <c r="D29">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B30" s="4">
+        <v>46136</v>
+      </c>
+      <c r="C30" t="s">
+        <v>195</v>
+      </c>
+      <c r="D30">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B31" s="4">
+        <v>46136</v>
+      </c>
+      <c r="C31" t="s">
+        <v>195</v>
+      </c>
+      <c r="D31">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -2660,7 +2930,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{901B77E3-1F91-4E2B-8B00-0170C6CF2EFB}">
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" customWidth="1"/>
@@ -2672,7 +2942,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -2684,15 +2954,15 @@
         <v>20</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>6</v>
@@ -2710,7 +2980,7 @@
         <v>40</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F2" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2719,7 +2989,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>14</v>
@@ -2737,7 +3007,7 @@
         <v>107</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F3" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2746,7 +3016,7 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>12</v>
@@ -2764,7 +3034,7 @@
         <v>72</v>
       </c>
       <c r="E4" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F4" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2773,7 +3043,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>8</v>
@@ -2791,7 +3061,7 @@
         <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F5" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2800,7 +3070,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>6</v>
@@ -2818,7 +3088,7 @@
         <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F6" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2827,7 +3097,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>14</v>
@@ -2845,7 +3115,7 @@
         <v>110</v>
       </c>
       <c r="E7" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F7" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2854,7 +3124,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>12</v>
@@ -2872,7 +3142,7 @@
         <v>79</v>
       </c>
       <c r="E8" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F8" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2881,7 +3151,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>8</v>
@@ -2899,7 +3169,7 @@
         <v>69</v>
       </c>
       <c r="E9" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F9" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2908,7 +3178,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="2" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B10" t="s">
         <v>8</v>
@@ -2926,7 +3196,7 @@
         <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F10" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2935,7 +3205,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="2" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B11" t="s">
         <v>16</v>
@@ -2953,7 +3223,7 @@
         <v>126</v>
       </c>
       <c r="E11" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F11" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2962,7 +3232,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="2" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
@@ -2980,7 +3250,7 @@
         <v>104</v>
       </c>
       <c r="E12" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F12" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -2989,7 +3259,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="2" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B13" t="s">
         <v>12</v>
@@ -3007,7 +3277,7 @@
         <v>83</v>
       </c>
       <c r="E13" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F13" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3016,7 +3286,7 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
@@ -3034,7 +3304,7 @@
         <v>77</v>
       </c>
       <c r="E14" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F14" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3043,7 +3313,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B15" t="s">
         <v>10</v>
@@ -3061,7 +3331,7 @@
         <v>104</v>
       </c>
       <c r="E15" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F15" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3070,7 +3340,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
@@ -3088,7 +3358,7 @@
         <v>126</v>
       </c>
       <c r="E16" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F16" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3097,7 +3367,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
@@ -3115,7 +3385,7 @@
         <v>107</v>
       </c>
       <c r="E17" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F17" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3124,7 +3394,7 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="2" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B18" t="s">
         <v>10</v>
@@ -3142,7 +3412,7 @@
         <v>92</v>
       </c>
       <c r="E18" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F18" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3151,7 +3421,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="2" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B19" t="s">
         <v>12</v>
@@ -3169,7 +3439,7 @@
         <v>74</v>
       </c>
       <c r="E19" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F19" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3178,7 +3448,7 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="2" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B20" t="s">
         <v>16</v>
@@ -3196,7 +3466,7 @@
         <v>126</v>
       </c>
       <c r="E20" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F20" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3205,7 +3475,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="2" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
@@ -3223,7 +3493,7 @@
         <v>61</v>
       </c>
       <c r="E21" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F21" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3232,7 +3502,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="B22" t="s">
         <v>6</v>
@@ -3250,7 +3520,7 @@
         <v>37</v>
       </c>
       <c r="E22" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F22" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3259,7 +3529,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="B23" t="s">
         <v>8</v>
@@ -3277,7 +3547,7 @@
         <v>57</v>
       </c>
       <c r="E23" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F23" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3286,7 +3556,7 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
@@ -3304,7 +3574,7 @@
         <v>107</v>
       </c>
       <c r="E24" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F24" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3313,7 +3583,7 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="B25" t="s">
         <v>12</v>
@@ -3331,7 +3601,7 @@
         <v>86</v>
       </c>
       <c r="E25" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F25" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3340,7 +3610,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="B26" t="s">
         <v>6</v>
@@ -3358,7 +3628,7 @@
         <v>34</v>
       </c>
       <c r="E26" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F26" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3367,7 +3637,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="B27" t="s">
         <v>12</v>
@@ -3385,7 +3655,7 @@
         <v>81</v>
       </c>
       <c r="E27" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F27" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3394,7 +3664,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="B28" t="s">
         <v>16</v>
@@ -3412,7 +3682,7 @@
         <v>126</v>
       </c>
       <c r="E28" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F28" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3421,7 +3691,7 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
@@ -3439,7 +3709,7 @@
         <v>110</v>
       </c>
       <c r="E29" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F29" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3448,7 +3718,7 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="2" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="B30" t="s">
         <v>8</v>
@@ -3466,7 +3736,7 @@
         <v>59</v>
       </c>
       <c r="E30" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F30" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3475,7 +3745,7 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="2" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="B31" t="s">
         <v>10</v>
@@ -3493,7 +3763,7 @@
         <v>89</v>
       </c>
       <c r="E31" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F31" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3502,7 +3772,7 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="2" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
@@ -3520,7 +3790,7 @@
         <v>61</v>
       </c>
       <c r="E32" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F32" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3529,7 +3799,7 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="2" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="B33" t="s">
         <v>12</v>
@@ -3547,7 +3817,7 @@
         <v>74</v>
       </c>
       <c r="E33" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F33" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3556,7 +3826,7 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="2" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="B34" t="s">
         <v>6</v>
@@ -3574,7 +3844,7 @@
         <v>128</v>
       </c>
       <c r="E34" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F34" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3583,7 +3853,7 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="2" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="B35" t="s">
         <v>12</v>
@@ -3601,7 +3871,7 @@
         <v>131</v>
       </c>
       <c r="E35" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F35" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3610,7 +3880,7 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="2" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
@@ -3628,7 +3898,7 @@
         <v>107</v>
       </c>
       <c r="E36" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F36" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3637,7 +3907,7 @@
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="2" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="B37" t="s">
         <v>8</v>
@@ -3655,7 +3925,7 @@
         <v>52</v>
       </c>
       <c r="E37" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F37" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3664,7 +3934,7 @@
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="2" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="B38" t="s">
         <v>6</v>
@@ -3682,7 +3952,7 @@
         <v>128</v>
       </c>
       <c r="E38" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F38" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3691,7 +3961,7 @@
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="2" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="B39" t="s">
         <v>12</v>
@@ -3709,7 +3979,7 @@
         <v>131</v>
       </c>
       <c r="E39" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F39" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3718,7 +3988,7 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="2" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="B40" t="s">
         <v>8</v>
@@ -3736,7 +4006,7 @@
         <v>64</v>
       </c>
       <c r="E40" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F40" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3745,7 +4015,7 @@
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="2" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="B41" t="s">
         <v>14</v>
@@ -3763,7 +4033,7 @@
         <v>110</v>
       </c>
       <c r="E41" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F41" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3772,7 +4042,7 @@
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="B42" t="s">
         <v>10</v>
@@ -3790,7 +4060,7 @@
         <v>95</v>
       </c>
       <c r="E42" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F42" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3799,7 +4069,7 @@
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="B43" t="s">
         <v>12</v>
@@ -3817,7 +4087,7 @@
         <v>131</v>
       </c>
       <c r="E43" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F43" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3826,7 +4096,7 @@
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="B44" t="s">
         <v>8</v>
@@ -3844,7 +4114,7 @@
         <v>57</v>
       </c>
       <c r="E44" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F44" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3853,7 +4123,7 @@
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="B45" t="s">
         <v>14</v>
@@ -3871,7 +4141,7 @@
         <v>107</v>
       </c>
       <c r="E45" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F45" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3880,7 +4150,7 @@
     </row>
     <row r="46" spans="1:6">
       <c r="A46" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B46" t="s">
         <v>10</v>
@@ -3898,7 +4168,7 @@
         <v>98</v>
       </c>
       <c r="E46" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F46" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3907,7 +4177,7 @@
     </row>
     <row r="47" spans="1:6">
       <c r="A47" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B47" t="s">
         <v>12</v>
@@ -3925,7 +4195,7 @@
         <v>77</v>
       </c>
       <c r="E47" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F47" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3934,7 +4204,7 @@
     </row>
     <row r="48" spans="1:6">
       <c r="A48" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B48" t="s">
         <v>8</v>
@@ -3952,7 +4222,7 @@
         <v>134</v>
       </c>
       <c r="E48" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F48" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3961,7 +4231,7 @@
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="B49" t="s">
         <v>14</v>
@@ -3979,7 +4249,7 @@
         <v>110</v>
       </c>
       <c r="E49" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F49" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -3988,7 +4258,7 @@
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="2" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B50" t="s">
         <v>10</v>
@@ -4006,7 +4276,7 @@
         <v>89</v>
       </c>
       <c r="E50" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F50" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4015,7 +4285,7 @@
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="2" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B51" t="s">
         <v>12</v>
@@ -4033,7 +4303,7 @@
         <v>74</v>
       </c>
       <c r="E51" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F51" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4042,7 +4312,7 @@
     </row>
     <row r="52" spans="1:6">
       <c r="A52" s="2" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B52" t="s">
         <v>8</v>
@@ -4060,7 +4330,7 @@
         <v>59</v>
       </c>
       <c r="E52" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F52" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4069,7 +4339,7 @@
     </row>
     <row r="53" spans="1:6">
       <c r="A53" s="2" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B53" t="s">
         <v>14</v>
@@ -4087,7 +4357,7 @@
         <v>114</v>
       </c>
       <c r="E53" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F53" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4096,7 +4366,7 @@
     </row>
     <row r="54" spans="1:6">
       <c r="A54" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="B54" t="s">
         <v>10</v>
@@ -4114,7 +4384,7 @@
         <v>89</v>
       </c>
       <c r="E54" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F54" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4123,7 +4393,7 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="B55" t="s">
         <v>12</v>
@@ -4141,7 +4411,7 @@
         <v>72</v>
       </c>
       <c r="E55" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F55" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4150,7 +4420,7 @@
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="B56" t="s">
         <v>8</v>
@@ -4168,7 +4438,7 @@
         <v>59</v>
       </c>
       <c r="E56" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F56" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4177,7 +4447,7 @@
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="B57" t="s">
         <v>14</v>
@@ -4195,7 +4465,7 @@
         <v>114</v>
       </c>
       <c r="E57" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F57" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4204,7 +4474,7 @@
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="2" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="B58" t="s">
         <v>10</v>
@@ -4222,7 +4492,7 @@
         <v>137</v>
       </c>
       <c r="E58" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F58" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4231,7 +4501,7 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="2" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="B59" t="s">
         <v>12</v>
@@ -4249,7 +4519,7 @@
         <v>137</v>
       </c>
       <c r="E59" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F59" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4258,7 +4528,7 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="2" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="B60" t="s">
         <v>8</v>
@@ -4276,7 +4546,7 @@
         <v>52</v>
       </c>
       <c r="E60" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F60" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4285,7 +4555,7 @@
     </row>
     <row r="61" spans="1:6">
       <c r="A61" s="2" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="B61" t="s">
         <v>14</v>
@@ -4303,7 +4573,7 @@
         <v>114</v>
       </c>
       <c r="E61" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F61" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4312,7 +4582,7 @@
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="2" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="B62" t="s">
         <v>10</v>
@@ -4330,7 +4600,7 @@
         <v>137</v>
       </c>
       <c r="E62" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F62" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4339,7 +4609,7 @@
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="2" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="B63" t="s">
         <v>12</v>
@@ -4357,7 +4627,7 @@
         <v>131</v>
       </c>
       <c r="E63" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F63" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4366,7 +4636,7 @@
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="2" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="B64" t="s">
         <v>8</v>
@@ -4384,7 +4654,7 @@
         <v>137</v>
       </c>
       <c r="E64" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F64" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4393,7 +4663,7 @@
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="2" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="B65" t="s">
         <v>14</v>
@@ -4411,7 +4681,7 @@
         <v>61</v>
       </c>
       <c r="E65" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F65" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4420,7 +4690,7 @@
     </row>
     <row r="66" spans="1:6">
       <c r="A66" s="2" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="B66" t="s">
         <v>10</v>
@@ -4438,7 +4708,7 @@
         <v>104</v>
       </c>
       <c r="E66" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F66" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4447,7 +4717,7 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" s="2" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="B67" t="s">
         <v>12</v>
@@ -4465,7 +4735,7 @@
         <v>81</v>
       </c>
       <c r="E67" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F67" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4474,7 +4744,7 @@
     </row>
     <row r="68" spans="1:6">
       <c r="A68" s="2" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="B68" t="s">
         <v>8</v>
@@ -4492,7 +4762,7 @@
         <v>61</v>
       </c>
       <c r="E68" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F68" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4501,7 +4771,7 @@
     </row>
     <row r="69" spans="1:6">
       <c r="A69" s="2" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="B69" t="s">
         <v>14</v>
@@ -4519,7 +4789,7 @@
         <v>110</v>
       </c>
       <c r="E69" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F69" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4528,7 +4798,7 @@
     </row>
     <row r="70" spans="1:6">
       <c r="A70" s="2" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="B70" t="s">
         <v>12</v>
@@ -4546,7 +4816,7 @@
         <v>131</v>
       </c>
       <c r="E70" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F70" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4555,7 +4825,7 @@
     </row>
     <row r="71" spans="1:6">
       <c r="A71" s="2" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="B71" t="s">
         <v>6</v>
@@ -4573,7 +4843,7 @@
         <v>128</v>
       </c>
       <c r="E71" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F71" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4582,7 +4852,7 @@
     </row>
     <row r="72" spans="1:6">
       <c r="A72" s="2" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="B72" t="s">
         <v>14</v>
@@ -4600,7 +4870,7 @@
         <v>107</v>
       </c>
       <c r="E72" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F72" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4609,7 +4879,7 @@
     </row>
     <row r="73" spans="1:6">
       <c r="A73" s="2" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="B73" t="s">
         <v>8</v>
@@ -4627,7 +4897,7 @@
         <v>66</v>
       </c>
       <c r="E73" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F73" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4636,7 +4906,7 @@
     </row>
     <row r="74" spans="1:6">
       <c r="A74" s="2" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="B74" t="s">
         <v>12</v>
@@ -4654,7 +4924,7 @@
         <v>77</v>
       </c>
       <c r="E74" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F74" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4663,7 +4933,7 @@
     </row>
     <row r="75" spans="1:6">
       <c r="A75" s="2" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="B75" t="s">
         <v>6</v>
@@ -4681,7 +4951,7 @@
         <v>25</v>
       </c>
       <c r="E75" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F75" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4690,7 +4960,7 @@
     </row>
     <row r="76" spans="1:6">
       <c r="A76" s="2" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="B76" t="s">
         <v>14</v>
@@ -4708,7 +4978,7 @@
         <v>61</v>
       </c>
       <c r="E76" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F76" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4717,7 +4987,7 @@
     </row>
     <row r="77" spans="1:6">
       <c r="A77" s="2" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="B77" t="s">
         <v>8</v>
@@ -4735,7 +5005,7 @@
         <v>46</v>
       </c>
       <c r="E77" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F77" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4744,7 +5014,7 @@
     </row>
     <row r="78" spans="1:6">
       <c r="A78" s="2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="B78" t="s">
         <v>6</v>
@@ -4762,7 +5032,7 @@
         <v>128</v>
       </c>
       <c r="E78" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F78" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4771,7 +5041,7 @@
     </row>
     <row r="79" spans="1:6">
       <c r="A79" s="2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="B79" t="s">
         <v>14</v>
@@ -4789,7 +5059,7 @@
         <v>107</v>
       </c>
       <c r="E79" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F79" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4798,7 +5068,7 @@
     </row>
     <row r="80" spans="1:6">
       <c r="A80" s="2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="B80" t="s">
         <v>12</v>
@@ -4816,7 +5086,7 @@
         <v>72</v>
       </c>
       <c r="E80" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F80" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4825,7 +5095,7 @@
     </row>
     <row r="81" spans="1:6">
       <c r="A81" s="2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="B81" t="s">
         <v>18</v>
@@ -4843,7 +5113,7 @@
         <v>123</v>
       </c>
       <c r="E81" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F81" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4852,7 +5122,7 @@
     </row>
     <row r="82" spans="1:6">
       <c r="A82" s="2" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="B82" t="s">
         <v>6</v>
@@ -4870,7 +5140,7 @@
         <v>25</v>
       </c>
       <c r="E82" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F82" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4879,7 +5149,7 @@
     </row>
     <row r="83" spans="1:6">
       <c r="A83" s="2" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="B83" t="s">
         <v>12</v>
@@ -4897,7 +5167,7 @@
         <v>79</v>
       </c>
       <c r="E83" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F83" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4906,7 +5176,7 @@
     </row>
     <row r="84" spans="1:6">
       <c r="A84" s="2" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="B84" t="s">
         <v>18</v>
@@ -4924,7 +5194,7 @@
         <v>123</v>
       </c>
       <c r="E84" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="F84" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
@@ -4933,7 +5203,7 @@
     </row>
     <row r="85" spans="1:6">
       <c r="A85" s="2" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="B85" t="s">
         <v>14</v>
@@ -4951,17 +5221,989 @@
         <v>114</v>
       </c>
       <c r="E85" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="F85" s="2">
         <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
         <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6">
+      <c r="A86" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B86" t="s">
+        <v>6</v>
+      </c>
+      <c r="C86" t="str" cm="1">
+        <f t="array" ref="C86">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D40</v>
+      </c>
+      <c r="D86" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="E86" t="s">
+        <v>202</v>
+      </c>
+      <c r="F86" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6">
+      <c r="A87" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B87" t="s">
+        <v>14</v>
+      </c>
+      <c r="C87" t="str" cm="1">
+        <f t="array" ref="C87">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D33</v>
+      </c>
+      <c r="D87" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E87" t="s">
+        <v>202</v>
+      </c>
+      <c r="F87" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6">
+      <c r="A88" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B88" t="s">
+        <v>12</v>
+      </c>
+      <c r="C88" t="str" cm="1">
+        <f t="array" ref="C88">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D41</v>
+      </c>
+      <c r="D88" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="E88" t="s">
+        <v>203</v>
+      </c>
+      <c r="F88" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6">
+      <c r="A89" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B89" t="s">
+        <v>18</v>
+      </c>
+      <c r="C89" t="str" cm="1">
+        <f t="array" ref="C89">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D49</v>
+      </c>
+      <c r="D89" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E89" t="s">
+        <v>202</v>
+      </c>
+      <c r="F89" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6">
+      <c r="A90" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B90" t="s">
+        <v>6</v>
+      </c>
+      <c r="C90" t="str" cm="1">
+        <f t="array" ref="C90">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D4</v>
+      </c>
+      <c r="D90" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E90" t="s">
+        <v>202</v>
+      </c>
+      <c r="F90" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6">
+      <c r="A91" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B91" t="s">
+        <v>14</v>
+      </c>
+      <c r="C91" t="str" cm="1">
+        <f t="array" ref="C91">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D32</v>
+      </c>
+      <c r="D91" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E91" t="s">
+        <v>202</v>
+      </c>
+      <c r="F91" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6">
+      <c r="A92" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B92" t="s">
+        <v>12</v>
+      </c>
+      <c r="C92" t="str" cm="1">
+        <f t="array" ref="C92">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D22</v>
+      </c>
+      <c r="D92" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E92" t="s">
+        <v>202</v>
+      </c>
+      <c r="F92" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6">
+      <c r="A93" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B93" t="s">
+        <v>18</v>
+      </c>
+      <c r="C93" t="str" cm="1">
+        <f t="array" ref="C93">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D49</v>
+      </c>
+      <c r="D93" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E93" t="s">
+        <v>203</v>
+      </c>
+      <c r="F93" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6">
+      <c r="A94" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B94" t="s">
+        <v>12</v>
+      </c>
+      <c r="C94" t="str" cm="1">
+        <f t="array" ref="C94">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D20</v>
+      </c>
+      <c r="D94" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E94" t="s">
+        <v>202</v>
+      </c>
+      <c r="F94" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6">
+      <c r="A95" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B95" t="s">
+        <v>6</v>
+      </c>
+      <c r="C95" t="str" cm="1">
+        <f t="array" ref="C95">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D40</v>
+      </c>
+      <c r="D95" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="E95" t="s">
+        <v>203</v>
+      </c>
+      <c r="F95" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6">
+      <c r="A96" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B96" t="s">
+        <v>18</v>
+      </c>
+      <c r="C96" t="str" cm="1">
+        <f t="array" ref="C96">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D50</v>
+      </c>
+      <c r="D96" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="E96" t="s">
+        <v>202</v>
+      </c>
+      <c r="F96" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6">
+      <c r="A97" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B97" t="s">
+        <v>14</v>
+      </c>
+      <c r="C97" t="str" cm="1">
+        <f t="array" ref="C97">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D32</v>
+      </c>
+      <c r="D97" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E97" t="s">
+        <v>202</v>
+      </c>
+      <c r="F97" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6">
+      <c r="A98" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B98" t="s">
+        <v>12</v>
+      </c>
+      <c r="C98" t="str" cm="1">
+        <f t="array" ref="C98">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D24</v>
+      </c>
+      <c r="D98" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E98" t="s">
+        <v>202</v>
+      </c>
+      <c r="F98" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6">
+      <c r="A99" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B99" t="s">
+        <v>6</v>
+      </c>
+      <c r="C99" t="str" cm="1">
+        <f t="array" ref="C99">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D2</v>
+      </c>
+      <c r="D99" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E99" t="s">
+        <v>202</v>
+      </c>
+      <c r="F99" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6">
+      <c r="A100" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B100" t="s">
+        <v>14</v>
+      </c>
+      <c r="C100" t="str" cm="1">
+        <f t="array" ref="C100">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D51</v>
+      </c>
+      <c r="D100" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E100" t="s">
+        <v>202</v>
+      </c>
+      <c r="F100" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6">
+      <c r="A101" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B101" t="s">
+        <v>18</v>
+      </c>
+      <c r="C101" t="str" cm="1">
+        <f t="array" ref="C101">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D50</v>
+      </c>
+      <c r="D101" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="E101" t="s">
+        <v>203</v>
+      </c>
+      <c r="F101" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6">
+      <c r="A102" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B102" t="s">
+        <v>12</v>
+      </c>
+      <c r="C102" t="str" cm="1">
+        <f t="array" ref="C102">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D23</v>
+      </c>
+      <c r="D102" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E102" t="s">
+        <v>202</v>
+      </c>
+      <c r="F102" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6">
+      <c r="A103" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B103" t="s">
+        <v>6</v>
+      </c>
+      <c r="C103" t="str" cm="1">
+        <f t="array" ref="C103">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D3</v>
+      </c>
+      <c r="D103" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E103" t="s">
+        <v>203</v>
+      </c>
+      <c r="F103" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6">
+      <c r="A104" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B104" t="s">
+        <v>14</v>
+      </c>
+      <c r="C104" t="str" cm="1">
+        <f t="array" ref="C104">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D51</v>
+      </c>
+      <c r="D104" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E104" t="s">
+        <v>202</v>
+      </c>
+      <c r="F104" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6">
+      <c r="A105" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B105" t="s">
+        <v>18</v>
+      </c>
+      <c r="C105" t="str" cm="1">
+        <f t="array" ref="C105">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D50</v>
+      </c>
+      <c r="D105" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="E105" t="s">
+        <v>202</v>
+      </c>
+      <c r="F105" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6">
+      <c r="A106" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B106" t="s">
+        <v>8</v>
+      </c>
+      <c r="C106" t="str" cm="1">
+        <f t="array" ref="C106">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D14</v>
+      </c>
+      <c r="D106" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E106" t="s">
+        <v>203</v>
+      </c>
+      <c r="F106" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6">
+      <c r="A107" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B107" t="s">
+        <v>10</v>
+      </c>
+      <c r="C107" t="str" cm="1">
+        <f t="array" ref="C107">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D45</v>
+      </c>
+      <c r="D107" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E107" t="s">
+        <v>202</v>
+      </c>
+      <c r="F107" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6">
+      <c r="A108" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B108" t="s">
+        <v>14</v>
+      </c>
+      <c r="C108" t="str" cm="1">
+        <f t="array" ref="C108">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D51</v>
+      </c>
+      <c r="D108" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E108" t="s">
+        <v>202</v>
+      </c>
+      <c r="F108" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6">
+      <c r="A109" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B109" t="s">
+        <v>12</v>
+      </c>
+      <c r="C109" t="str" cm="1">
+        <f t="array" ref="C109">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D52</v>
+      </c>
+      <c r="D109" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="E109" t="s">
+        <v>202</v>
+      </c>
+      <c r="F109" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6">
+      <c r="A110" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B110" t="s">
+        <v>8</v>
+      </c>
+      <c r="C110" t="str" cm="1">
+        <f t="array" ref="C110">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D12</v>
+      </c>
+      <c r="D110" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E110" t="s">
+        <v>203</v>
+      </c>
+      <c r="F110" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6">
+      <c r="A111" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B111" t="s">
+        <v>10</v>
+      </c>
+      <c r="C111" t="str" cm="1">
+        <f t="array" ref="C111">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D30</v>
+      </c>
+      <c r="D111" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E111" t="s">
+        <v>202</v>
+      </c>
+      <c r="F111" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6">
+      <c r="A112" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B112" t="s">
+        <v>14</v>
+      </c>
+      <c r="C112" t="str" cm="1">
+        <f t="array" ref="C112">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D51</v>
+      </c>
+      <c r="D112" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E112" t="s">
+        <v>202</v>
+      </c>
+      <c r="F112" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6">
+      <c r="A113" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B113" t="s">
+        <v>12</v>
+      </c>
+      <c r="C113" t="str" cm="1">
+        <f t="array" ref="C113">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D41</v>
+      </c>
+      <c r="D113" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="E113" t="s">
+        <v>202</v>
+      </c>
+      <c r="F113" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6">
+      <c r="A114" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B114" t="s">
+        <v>8</v>
+      </c>
+      <c r="C114" t="str" cm="1">
+        <f t="array" ref="C114">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D53</v>
+      </c>
+      <c r="D114" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="E114" t="s">
+        <v>203</v>
+      </c>
+      <c r="F114" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6">
+      <c r="A115" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B115" t="s">
+        <v>10</v>
+      </c>
+      <c r="C115" t="str" cm="1">
+        <f t="array" ref="C115">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D27</v>
+      </c>
+      <c r="D115" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E115" t="s">
+        <v>202</v>
+      </c>
+      <c r="F115" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6">
+      <c r="A116" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B116" t="s">
+        <v>14</v>
+      </c>
+      <c r="C116" t="str" cm="1">
+        <f t="array" ref="C116">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D32</v>
+      </c>
+      <c r="D116" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E116" t="s">
+        <v>202</v>
+      </c>
+      <c r="F116" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6">
+      <c r="A117" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B117" t="s">
+        <v>12</v>
+      </c>
+      <c r="C117" t="str" cm="1">
+        <f t="array" ref="C117">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D23</v>
+      </c>
+      <c r="D117" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E117" t="s">
+        <v>202</v>
+      </c>
+      <c r="F117" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6">
+      <c r="A118" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B118" t="s">
+        <v>8</v>
+      </c>
+      <c r="C118" t="str" cm="1">
+        <f t="array" ref="C118">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D13</v>
+      </c>
+      <c r="D118" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E118" t="s">
+        <v>203</v>
+      </c>
+      <c r="F118" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6">
+      <c r="A119" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B119" t="s">
+        <v>10</v>
+      </c>
+      <c r="C119" t="str" cm="1">
+        <f t="array" ref="C119">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D25</v>
+      </c>
+      <c r="D119" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E119" t="s">
+        <v>202</v>
+      </c>
+      <c r="F119" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6">
+      <c r="A120" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B120" t="s">
+        <v>14</v>
+      </c>
+      <c r="C120" t="str" cm="1">
+        <f t="array" ref="C120">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D32</v>
+      </c>
+      <c r="D120" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E120" t="s">
+        <v>202</v>
+      </c>
+      <c r="F120" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6">
+      <c r="A121" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B121" t="s">
+        <v>12</v>
+      </c>
+      <c r="C121" t="str" cm="1">
+        <f t="array" ref="C121">_xlfn.XLOOKUP(1,
+   (tblDecks[Commander]=tblGamePlayers[[#This Row],[Commander]])*
+   (tblDecks[PlayerName]=tblGamePlayers[[#This Row],[PlayerName]]),
+   tblDecks[DeckID],
+   ""
+)</f>
+        <v>D19</v>
+      </c>
+      <c r="D121" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E121" t="s">
+        <v>202</v>
+      </c>
+      <c r="F121" s="2">
+        <f>IF(tblGamePlayers[[#This Row],[Result]]="Win",1,0)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B85" xr:uid="{8681415D-26E5-48F3-B990-4324A23F1CFB}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B121" xr:uid="{8681415D-26E5-48F3-B990-4324A23F1CFB}">
       <formula1>PlayerList</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{86E4FB70-4529-47DF-A939-BD41AD4D0FA0}">
@@ -4977,7 +6219,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2FAD5EF-FA4E-4366-BDF6-EE476BE4A0C0}">
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.7109375" customWidth="1"/>
@@ -4999,16 +6241,16 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>180</v>
+        <v>204</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>181</v>
+        <v>205</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>182</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -5054,7 +6296,7 @@
       </c>
       <c r="D3">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5062,7 +6304,7 @@
       </c>
       <c r="F3">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5083,11 +6325,11 @@
       </c>
       <c r="D4">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
@@ -5095,7 +6337,7 @@
       </c>
       <c r="G4" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -5112,7 +6354,7 @@
       </c>
       <c r="D5">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5120,11 +6362,11 @@
       </c>
       <c r="F5">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -5344,11 +6586,11 @@
       </c>
       <c r="D13">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
@@ -5356,7 +6598,7 @@
       </c>
       <c r="G13" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0.5</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -5373,11 +6615,11 @@
       </c>
       <c r="D14">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
@@ -5385,7 +6627,7 @@
       </c>
       <c r="G14" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0.66666666666666663</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -5402,11 +6644,11 @@
       </c>
       <c r="D15">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
@@ -5414,7 +6656,7 @@
       </c>
       <c r="G15" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -5547,7 +6789,7 @@
       </c>
       <c r="D20">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E20">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5555,11 +6797,11 @@
       </c>
       <c r="F20">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G20" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0.33333333333333331</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -5576,7 +6818,7 @@
       </c>
       <c r="D21">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E21">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5584,7 +6826,7 @@
       </c>
       <c r="F21">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G21" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5634,7 +6876,7 @@
       </c>
       <c r="D23">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E23">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5642,7 +6884,7 @@
       </c>
       <c r="F23">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G23" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5663,7 +6905,7 @@
       </c>
       <c r="D24">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E24">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5671,7 +6913,7 @@
       </c>
       <c r="F24">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G24" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5692,7 +6934,7 @@
       </c>
       <c r="D25">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5700,7 +6942,7 @@
       </c>
       <c r="F25">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G25" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5721,7 +6963,7 @@
       </c>
       <c r="D26">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E26">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5729,7 +6971,7 @@
       </c>
       <c r="F26">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G26" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5779,7 +7021,7 @@
       </c>
       <c r="D28">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5787,7 +7029,7 @@
       </c>
       <c r="F28">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G28" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -5866,7 +7108,7 @@
       </c>
       <c r="D31">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5874,11 +7116,11 @@
       </c>
       <c r="F31">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G31" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0.33333333333333331</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -5924,7 +7166,7 @@
       </c>
       <c r="D33">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E33">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5932,11 +7174,11 @@
       </c>
       <c r="F33">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G33" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0.2</v>
+        <v>0.1111111111111111</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -5953,7 +7195,7 @@
       </c>
       <c r="D34">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E34">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -5961,7 +7203,7 @@
       </c>
       <c r="F34">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G34" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
@@ -6157,19 +7399,19 @@
       </c>
       <c r="D41">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E41">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F41">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G41" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -6186,19 +7428,19 @@
       </c>
       <c r="D42">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E42">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F42">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G42" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0.2</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -6302,7 +7544,7 @@
       </c>
       <c r="D46" s="7">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E46" s="7">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
@@ -6310,11 +7552,11 @@
       </c>
       <c r="F46" s="7">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G46" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -6418,19 +7660,135 @@
       </c>
       <c r="D50" s="7">
         <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E50" s="7">
         <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50" s="7">
         <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G50" s="6">
         <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
-        <v>0</v>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B51" s="7" t="str">
+        <f>_xlfn.XLOOKUP(tblDeckDashboard[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[Commander], "")</f>
+        <v>Mister Negative</v>
+      </c>
+      <c r="C51" s="7" t="str">
+        <f>_xlfn.XLOOKUP(tblDeckDashboard[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[PlayerName], "")</f>
+        <v>Jon Paul</v>
+      </c>
+      <c r="D51" s="7">
+        <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
+        <v>3</v>
+      </c>
+      <c r="E51" s="7">
+        <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
+        <v>1</v>
+      </c>
+      <c r="F51" s="7">
+        <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
+        <v>2</v>
+      </c>
+      <c r="G51" s="6">
+        <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B52" s="7" t="str">
+        <f>_xlfn.XLOOKUP(tblDeckDashboard[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[Commander], "")</f>
+        <v>Bria, Riptide Rogue</v>
+      </c>
+      <c r="C52" s="7" t="str">
+        <f>_xlfn.XLOOKUP(tblDeckDashboard[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[PlayerName], "")</f>
+        <v>Mark</v>
+      </c>
+      <c r="D52" s="7">
+        <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
+        <v>4</v>
+      </c>
+      <c r="E52" s="7">
+        <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
+        <v>0</v>
+      </c>
+      <c r="F52" s="7">
+        <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
+        <v>4</v>
+      </c>
+      <c r="G52" s="6">
+        <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="A53" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B53" s="7" t="str">
+        <f>_xlfn.XLOOKUP(tblDeckDashboard[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[Commander], "")</f>
+        <v>Dina, Essence Brewer</v>
+      </c>
+      <c r="C53" s="7" t="str">
+        <f>_xlfn.XLOOKUP(tblDeckDashboard[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[PlayerName], "")</f>
+        <v>Chavez</v>
+      </c>
+      <c r="D53" s="7">
+        <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
+        <v>1</v>
+      </c>
+      <c r="E53" s="7">
+        <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
+        <v>0</v>
+      </c>
+      <c r="F53" s="7">
+        <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
+        <v>1</v>
+      </c>
+      <c r="G53" s="6">
+        <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B54" s="7" t="str">
+        <f>_xlfn.XLOOKUP(tblDeckDashboard[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[Commander], "")</f>
+        <v>Nashi, Moon Sage's Scion</v>
+      </c>
+      <c r="C54" s="7" t="str">
+        <f>_xlfn.XLOOKUP(tblDeckDashboard[[#This Row],[DeckID]], tblDecks[DeckID], tblDecks[PlayerName], "")</f>
+        <v>Nick</v>
+      </c>
+      <c r="D54" s="7">
+        <f>COUNTIF(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]])</f>
+        <v>1</v>
+      </c>
+      <c r="E54" s="7">
+        <f>SUMIFS(tblGamePlayers[WinFlag], tblGamePlayers[DeckID], tblDeckDashboard[[#This Row],[DeckID]])</f>
+        <v>1</v>
+      </c>
+      <c r="F54" s="7">
+        <f>COUNTIFS(tblGamePlayers[DeckID],tblDeckDashboard[[#This Row],[DeckID]], tblGamePlayers[Result],"Loss*")</f>
+        <v>0</v>
+      </c>
+      <c r="G54" s="6">
+        <f>IF(tblDeckDashboard[[#This Row],[Total Games]]=0,0,tblDeckDashboard[[#This Row],[Wins]]/tblDeckDashboard[[#This Row],[Total Games]])</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>